<commit_message>
added function for adding a new row
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hulme\Desktop\it-equipment-inventory-management-system\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DD9A0A04-C2F9-403D-BC91-A3F8CBAF7DA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82FE09F4-2DF5-4EA6-B81E-751C5CE325B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{9D68D1CA-928C-419E-A018-B009A42BA13A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Device Name</t>
   </si>
@@ -72,6 +72,12 @@
   </si>
   <si>
     <t>test</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Repair</t>
   </si>
 </sst>
 </file>
@@ -444,7 +450,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47991ED3-0337-48B7-AD2F-A40CEA66B0E2}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.36328125" customWidth="1"/>
@@ -452,7 +458,7 @@
     <col min="5" max="5" width="10.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -471,8 +477,11 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -490,6 +499,9 @@
       </c>
       <c r="F2" t="s">
         <v>10</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added reindex to save function, after testing, I had an issue with the data not formatting correctly in excel
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -2,44 +2,25 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hulme\Desktop\it-equipment-inventory-management-system\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82FE09F4-2DF5-4EA6-B81E-751C5CE325B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1548C946-1DF3-489A-BAFC-CC531774E42A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{9D68D1CA-928C-419E-A018-B009A42BA13A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
   <si>
     <t>Device Name</t>
   </si>
@@ -50,45 +31,57 @@
     <t>User</t>
   </si>
   <si>
-    <t xml:space="preserve">Location </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Date </t>
+    <t>location</t>
+  </si>
+  <si>
+    <t>Date</t>
   </si>
   <si>
     <t>Notes</t>
   </si>
   <si>
-    <t>PC- 001</t>
-  </si>
-  <si>
-    <t>Desktop</t>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>PC02</t>
+  </si>
+  <si>
+    <t>desktop</t>
+  </si>
+  <si>
+    <t>Mark</t>
+  </si>
+  <si>
+    <t>Dairy</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>active</t>
+  </si>
+  <si>
+    <t>PC023</t>
   </si>
   <si>
     <t>Sam</t>
   </si>
   <si>
     <t>IT</t>
-  </si>
-  <si>
-    <t>test</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Repair</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -115,13 +108,13 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -144,44 +137,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -208,32 +201,14 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -260,24 +235,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -289,173 +246,175 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
-            <a:schemeClr val="phClr"/>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47991ED3-0337-48B7-AD2F-A40CEA66B0E2}">
-  <dimension ref="A1:G2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.36328125" customWidth="1"/>
-    <col min="2" max="2" width="11.1796875" customWidth="1"/>
-    <col min="5" max="5" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="48.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -478,33 +437,56 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E2" s="1">
-        <v>46145</v>
+        <v>46145.862742025463</v>
       </c>
       <c r="F2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G2" t="s">
         <v>12</v>
       </c>
     </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="1">
+        <v>46145.863119605623</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" t="s">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
addedsystem_info.py which collects system infomation automatically using powershell commands ready for main.py, bug fixes to main.py
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -1,94 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hulme\Desktop\it-equipment-inventory-management-system\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1548C946-1DF3-489A-BAFC-CC531774E42A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
-  <si>
-    <t>Device Name</t>
-  </si>
-  <si>
-    <t>Device Type</t>
-  </si>
-  <si>
-    <t>User</t>
-  </si>
-  <si>
-    <t>location</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>PC02</t>
-  </si>
-  <si>
-    <t>desktop</t>
-  </si>
-  <si>
-    <t>Mark</t>
-  </si>
-  <si>
-    <t>Dairy</t>
-  </si>
-  <si>
-    <t>test</t>
-  </si>
-  <si>
-    <t>active</t>
-  </si>
-  <si>
-    <t>PC023</t>
-  </si>
-  <si>
-    <t>Sam</t>
-  </si>
-  <si>
-    <t>IT</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
-  </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -106,23 +46,81 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -410,80 +408,207 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="5" max="5" width="48.453125" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Asset Tag</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Device Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Device Type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Serial Number</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Model Number</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>MAC Address</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="1">
-        <v>46145.862742025463</v>
-      </c>
-      <c r="F2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" t="s">
-        <v>12</v>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ASSET-0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Name         
+----         
+LCDLAPTOP1756</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>SystemType  
+----------  
+x64-based PC</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>SerialNumber
+------------
+CND2013YKD</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Model                
+-----                
+HP 250 G8 Notebook PC</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>MACAddress       
+----------       
+10:6F:D9:BD:C4:43</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>UserName         
+--------         
+CLAWSON\sam.hulme</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>05-09-2026</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>No notes</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="1">
-        <v>46145.863119605623</v>
-      </c>
-      <c r="F3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G3" t="s">
-        <v>12</v>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ASSET-0002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Name         
+----         
+LCDLAPTOP1756</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>SystemType  
+----------  
+x64-based PC</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>SerialNumber
+------------
+CND2013YKD</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Model                
+-----                
+HP 250 G8 Notebook PC</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>MACAddress       
+----------       
+10:6F:D9:BD:C4:43</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>UserName         
+--------         
+CLAWSON\sam.hulme</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>05-09-2026</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>No notes</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
worked on validation and edit functions
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -537,75 +537,6 @@
         </is>
       </c>
       <c r="K2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>ASSET-0002</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Name         
-----         
-LCDLAPTOP1756</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>SystemType  
-----------  
-x64-based PC</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>SerialNumber
-------------
-CND2013YKD</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Model                
------                
-HP 250 G8 Notebook PC</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>MACAddress       
-----------       
-10:6F:D9:BD:C4:43</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>UserName         
---------         
-CLAWSON\sam.hulme</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>05-09-2026</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>No notes</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>

</xml_diff>

<commit_message>
added to backups, now only store 10 saves, take out device now goes off asset tag which fixes bug with manual devices not being able to be checked out
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,6 +474,61 @@
       <c r="K1" t="inlineStr">
         <is>
           <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ASSET-000w</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>LCDLAPTOP1756</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>x64-based PC</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>CND2013YKD</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>HP 250 G8 Notebook PC</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>10:6F:D9:BD:C4:43</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>CLAWSON\sam.hulme</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="n">
+        <v>46154</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>No notes</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
changed device name to asset name for continuity with other excel docs, removed checkout function, outside the scope of this project, added config.py to fix file path errors when running off memory stick
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -428,7 +428,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Device Name</t>
+          <t>Asset Name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -480,7 +480,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ASSET-000w</t>
+          <t>ASSET-0001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -519,11 +519,11 @@
         </is>
       </c>
       <c r="I2" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>No notes</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">

</xml_diff>